<commit_message>
Support optional listing photos and property reels
</commit_message>
<xml_diff>
--- a/inventory-example.xlsx
+++ b/inventory-example.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory template" sheetId="1" r:id="R5b305243b7e344dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples only" sheetId="2" r:id="Rb7f7bb9be10e4658"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory template" sheetId="1" r:id="Rd744a78779054b18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples only" sheetId="2" r:id="R1904e60f508f4b42"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -307,6 +307,7 @@
     <x:col min="10" max="10" width="57" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="45" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="54" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -345,6 +346,9 @@
       </x:c>
       <x:c r="L1" s="3" t="str">
         <x:v>images</x:v>
+      </x:c>
+      <x:c r="M1" s="3" t="str">
+        <x:v>reel</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
@@ -360,6 +364,7 @@
       <x:c r="J2" s="6"/>
       <x:c r="K2" s="6"/>
       <x:c r="L2" s="6"/>
+      <x:c r="M2" s="6"/>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="6"/>
@@ -374,6 +379,7 @@
       <x:c r="J3" s="6"/>
       <x:c r="K3" s="6"/>
       <x:c r="L3" s="6"/>
+      <x:c r="M3" s="6"/>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
       <x:c r="A4" s="6"/>
@@ -388,6 +394,7 @@
       <x:c r="J4" s="6"/>
       <x:c r="K4" s="6"/>
       <x:c r="L4" s="6"/>
+      <x:c r="M4" s="6"/>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
       <x:c r="A5" s="6"/>
@@ -402,6 +409,7 @@
       <x:c r="J5" s="6"/>
       <x:c r="K5" s="6"/>
       <x:c r="L5" s="6"/>
+      <x:c r="M5" s="6"/>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="6"/>
@@ -416,6 +424,7 @@
       <x:c r="J6" s="6"/>
       <x:c r="K6" s="6"/>
       <x:c r="L6" s="6"/>
+      <x:c r="M6" s="6"/>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="6"/>
@@ -430,6 +439,7 @@
       <x:c r="J7" s="6"/>
       <x:c r="K7" s="6"/>
       <x:c r="L7" s="6"/>
+      <x:c r="M7" s="6"/>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="6"/>
@@ -444,6 +454,7 @@
       <x:c r="J8" s="6"/>
       <x:c r="K8" s="6"/>
       <x:c r="L8" s="6"/>
+      <x:c r="M8" s="6"/>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="6"/>
@@ -458,6 +469,7 @@
       <x:c r="J9" s="6"/>
       <x:c r="K9" s="6"/>
       <x:c r="L9" s="6"/>
+      <x:c r="M9" s="6"/>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="6"/>
@@ -472,6 +484,7 @@
       <x:c r="J10" s="6"/>
       <x:c r="K10" s="6"/>
       <x:c r="L10" s="6"/>
+      <x:c r="M10" s="6"/>
     </x:row>
     <x:row r="11">
       <x:c r="I11" s="8"/>
@@ -1081,6 +1094,7 @@
     <x:col min="10" max="10" width="57" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="45" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="54" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -1120,6 +1134,9 @@
       <x:c r="L1" s="3" t="str">
         <x:v>images</x:v>
       </x:c>
+      <x:c r="M1" s="3" t="str">
+        <x:v>reel</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -1156,7 +1173,10 @@
         <x:v>Balcony|Parking</x:v>
       </x:c>
       <x:c r="L2" s="6" t="str">
-        <x:v>https://example.com/approved-flat-photo.jpg</x:v>
+        <x:v>https://drive.google.com/file/d/PHOTO_ID_1/view|https://drive.google.com/file/d/PHOTO_ID_2/view</x:v>
+      </x:c>
+      <x:c r="M2" s="6" t="str">
+        <x:v>https://www.instagram.com/reel/SHORTCODE/</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
@@ -1192,6 +1212,7 @@
         <x:v>Ground floor|Road facing</x:v>
       </x:c>
       <x:c r="L3" s="6" t="str"/>
+      <x:c r="M3" s="6" t="str"/>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
       <x:c r="A4" s="6"/>
@@ -1206,6 +1227,7 @@
       <x:c r="J4" s="6"/>
       <x:c r="K4" s="6"/>
       <x:c r="L4" s="6"/>
+      <x:c r="M4" s="6"/>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
       <x:c r="A5" s="9" t="str">
@@ -1222,6 +1244,7 @@
       <x:c r="J5" s="6"/>
       <x:c r="K5" s="6"/>
       <x:c r="L5" s="6"/>
+      <x:c r="M5" s="6"/>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -1238,10 +1261,11 @@
       <x:c r="J6" s="6"/>
       <x:c r="K6" s="6"/>
       <x:c r="L6" s="6"/>
+      <x:c r="M6" s="6"/>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="9" t="str">
-        <x:v>Separate multiple features or photo URLs with |. Keep prices and private notes out of the shared workbook.</x:v>
+        <x:v>Separate multiple photo links with |. Images and reel are optional. Keep prices and private notes out of the shared workbook.</x:v>
       </x:c>
       <x:c r="B7" s="6"/>
       <x:c r="C7" s="6"/>
@@ -1254,6 +1278,7 @@
       <x:c r="J7" s="6"/>
       <x:c r="K7" s="6"/>
       <x:c r="L7" s="6"/>
+      <x:c r="M7" s="6"/>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="6"/>
@@ -1268,6 +1293,7 @@
       <x:c r="J8" s="6"/>
       <x:c r="K8" s="6"/>
       <x:c r="L8" s="6"/>
+      <x:c r="M8" s="6"/>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="6"/>
@@ -1282,6 +1308,7 @@
       <x:c r="J9" s="6"/>
       <x:c r="K9" s="6"/>
       <x:c r="L9" s="6"/>
+      <x:c r="M9" s="6"/>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="6"/>
@@ -1296,6 +1323,7 @@
       <x:c r="J10" s="6"/>
       <x:c r="K10" s="6"/>
       <x:c r="L10" s="6"/>
+      <x:c r="M10" s="6"/>
     </x:row>
     <x:row r="11">
       <x:c r="I11" s="8"/>

</xml_diff>